<commit_message>
Update Store Leader data and rename UP to Store Leader
Merge fresh Store Leader names/contacts from the September 2026
leader roster, remove one mislabeled Erablue store that had been
incorrectly tagged as Erafone in the source master data (120 stores
remain), and rename the "UP" label to "Store Leader" across the
dashboard UI, tag preview, and Excel export.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ERAFONE-STORE-LIST-SEPTEMBER-2026.xlsx
+++ b/ERAFONE-STORE-LIST-SEPTEMBER-2026.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I122"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Nama Store Leader</t>
+          <t>Store Leader</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -530,12 +530,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PANJI ARSY ARYA DILLAH</t>
+          <t>Panji Arsy Arya Dillah</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>+62 887-0770-0830</t>
+          <t>88707700830</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Achmad Fauzan</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87877698466</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Cahyo Suhendro</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85775411012</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dyah Laras Safitri</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>(021) 2528112</t>
+          <t>87872297994</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bagus Purbantoro</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>021-40127048</t>
+          <t>81517348893</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Erwin Ilyas</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>021-23581328</t>
+          <t>87776337231</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -890,12 +890,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Firman Saputra</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>021 42901379</t>
+          <t>81563259098</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Khoirul Amirudin</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>021 - 34832347</t>
+          <t>81380064450</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1115,12 +1115,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Citra Lusiana</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81292421449</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1160,12 +1160,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Roby Hidayat</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85788706963</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Adityo A Putra</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>82114003070</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1250,12 +1250,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rizki Maulana Sidiq</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85782953531</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1295,12 +1295,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Danang Setyawan</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89693534300</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Feri Tri Prabowo</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>021-541817</t>
+          <t>87807011995</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Alija Kalifa Akbar</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>021-5239-1560</t>
+          <t>81806161216</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Yasir</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85894016838</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Della Putri Fauza</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81213148340</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bagas Ajiyanto</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85156549329</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1655,12 +1655,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Habibie Al Ghazali</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>881024737300</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Asep Mulyana</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81908120555</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>HAMID SANUSI</t>
+          <t>Hamid Sanusi</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ananda Aulia Rochman</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87877603272</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1925,12 +1925,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Adit Sukma Anggara</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81351451449</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1970,12 +1970,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Fernaldhy Julian Sanusi</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8568622126</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2015,12 +2015,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Theodorus Eltara Ilvian Ristiawan</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>021 73471725</t>
+          <t>81617329666</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calisan</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81510282392</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Abdel Fickry Lain</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81112015550</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>RIKI NOVIANTO</t>
+          <t>Riki Novianto</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2330,12 +2330,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ma'ruf Wijaya</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>021 - 6310978</t>
+          <t>83807745664</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2465,12 +2465,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ridwan Rifaldo</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>021-5666845</t>
+          <t>81513629299</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2510,12 +2510,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rudi Noviansyah</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81919151192</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2555,12 +2555,12 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Sigit Dwi Anggoro</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85875091110</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2600,12 +2600,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Levia Suci Hardiyanti</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>82114852216</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Agung Kurniawan</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81519440612</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2690,12 +2690,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dyna Fitria</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8562000008</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2870,12 +2870,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Muhamad Igfir Refi Syarip</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>895395257767</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Diyanti</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89615673553</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Iqbal Firdaus</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85959388797</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3050,12 +3050,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Muhamad Igfir Refi Syarip</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>895395257767</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3095,12 +3095,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Muhammad Riduan Wahid</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89603352071</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Rama Prasetyo</t>
+          <t>Serpon</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3185,12 +3185,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rizki Tazakka</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81779941945</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3275,12 +3275,12 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Rama Prasetyo</t>
+          <t>Alfian</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>81291059132</t>
+          <t>85747292806</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3320,12 +3320,12 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Mochammad Ramdan Akbar</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85894568558</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3365,12 +3365,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Mulyana</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>021-59993809</t>
+          <t>87776764678</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3410,12 +3410,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Andri Sundara</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>021-59993587</t>
+          <t>81318321003</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3455,12 +3455,12 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rezky Nabila</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>+622159990668</t>
+          <t>89678086600</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3500,12 +3500,12 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Diki Febriyanto</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>895363851554</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3545,12 +3545,12 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Niko</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>021-54213507</t>
+          <t>87771807710</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>+62 877-7083-6816</t>
+          <t>87770836816</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -3680,12 +3680,12 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ramdani Andika Pramandana</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>82221833394</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3725,12 +3725,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Sugianto</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85888026212</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Elvirawati</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87880648402</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3815,12 +3815,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Aditya Anjasmara</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87778274871</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -3950,12 +3950,12 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Fahrul Yanuar</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8985500577</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -3995,12 +3995,12 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Teguh Prakoso</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81287162443</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -4085,12 +4085,12 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Irfan Supiandi</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81276004200</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Edi Suryadi</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85959594176</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>82124749133</t>
+          <t>81315592228</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4220,12 +4220,12 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Misbahul Badri</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81283260410</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -4265,12 +4265,12 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ade Rizky Pajarian</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81574755707</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -4400,12 +4400,12 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Muhammad Dendy</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81281736135</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -4445,12 +4445,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Mahfudin</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>816652158</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -4470,37 +4470,37 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>G546</t>
+          <t>M093</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>ERABLUE CILEDUG RAYA TANGERANG</t>
+          <t>MEGASTORE RUKO CIPONDOH TANGERANG</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Cukat Yoga Aditya</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89526719552</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Jl. Ciledug Raya No. 30 RT.006/RW.002, Petukangan Utara, Kec. Pesanggrahan, Kota Tangerang, Banten 15156</t>
+          <t>Jl KH Hasyim Asyhari RT003/RW003 No. 67B Cipondoh Tangerang</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -4515,12 +4515,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>M093</t>
+          <t>E290</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO CIPONDOH TANGERANG</t>
+          <t>ERAFONE FRANCHISE RUKO PORIS</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4530,22 +4530,22 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Cukat Yoga Aditya</t>
+          <t>Hasril Oktama</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>89526719552</t>
+          <t>8976118817</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Jl KH Hasyim Asyhari RT003/RW003 No. 67B Cipondoh Tangerang</t>
+          <t>Jalan Poris indah Raya, Ruko Paradise Eksklusif. Poris Gaga Batu Ceper Tangerang</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>E290</t>
+          <t>E646</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE FRANCHISE RUKO PORIS</t>
+          <t>ERAFONE BATU CEPER</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4575,22 +4575,22 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Saiful Zuhdi</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81284458691</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Jalan Poris indah Raya, Ruko Paradise Eksklusif. Poris Gaga Batu Ceper Tangerang</t>
+          <t>Jl. Halim Perdana Kusuma, RT.002/RW.001, Jurumudi Baru, Kec. Batuceper, Kota Tangerang, Banten 15122</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -4605,12 +4605,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>E646</t>
+          <t>E119</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE BATU CEPER</t>
+          <t>ERAFONE TANGERANG CITY MALL</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4625,17 +4625,17 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Saiful Zuhdi</t>
+          <t>Mega Nurhatifah, SE</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>81284458691</t>
+          <t>81284456745</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Jl. Halim Perdana Kusuma, RT.002/RW.001, Jurumudi Baru, Kec. Batuceper, Kota Tangerang, Banten 15122</t>
+          <t>Tangerang City Mall Lantai LG, Jl. Jenderal Sudirman No.1, RT.001/RW.005, Babakan, Kec. Tangerang, Kota Tangerang, Banten 15117</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -4650,12 +4650,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>E119</t>
+          <t>E696</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE TANGERANG CITY MALL</t>
+          <t>ERAFONE MB RASUNA SAID</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4665,22 +4665,22 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Mega Nurhatifah</t>
+          <t>Muhamad Riyanto</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>81284456745</t>
+          <t>87817170393</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Tangerang City Mall Lantai LG, Jl. Jenderal Sudirman No.1, RT.001/RW.005, Babakan, Kec. Tangerang, Kota Tangerang, Banten 15117</t>
+          <t>JL.HR Rasuna Said RT01/RW 02 Pakojan, kec.Pinang, Kota Tangerang, Banten 15142</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -4695,12 +4695,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>E696</t>
+          <t>M176</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB RASUNA SAID</t>
+          <t>ERAFONE AND MORE KISAMAUN</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -4710,22 +4710,22 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Muammar Alfis</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81212400080</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>JL.HR Rasuna Said RT01/RW 02 Pakojan, kec.Pinang, Kota Tangerang, Banten 15142</t>
+          <t>Jl Kisamaun No 89G RT/RW 002/007 Kel. Sukasari Kec. Tangerang Kota Tangerang</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
@@ -4740,12 +4740,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>M176</t>
+          <t>E422</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE KISAMAUN</t>
+          <t>ERAFONE RUKO M TOHA TANGERANG</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4755,22 +4755,22 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Muammar Alfis</t>
+          <t>Michael Roma Nelson</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>+62 812 1240 0080</t>
+          <t>81212456692</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Jl Kisamaun No 89G RT/RW 002/007 Kel. Sukasari Kec. Tangerang Kota Tangerang</t>
+          <t>Jl. Moh. Toha. RT 001/Rw.008 Pabuaran Tumpeng, Kec Karawaci, Kota Tangerang, 15114</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -4785,12 +4785,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>E422</t>
+          <t>M061</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO M TOHA TANGERANG</t>
+          <t>MEGASTORE RUKO JATIUWUNG</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4800,22 +4800,22 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Santo</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85813046313</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Jl. Moh. Toha. RT 001/Rw.008 Pabuaran Tumpeng, Kec Karawaci, Kota Tangerang, 15114</t>
+          <t>Jl. Gatot Subroto No. A1-A2 RT.001/RW.4, Sangiang Jaya, Kec. Periuk, Kota Tangerang, Banten 15134</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
@@ -4830,12 +4830,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>M061</t>
+          <t>E684</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO JATIUWUNG</t>
+          <t>ERAFONE RUKO SANGIANG TANGERANG</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4845,22 +4845,22 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Santo</t>
+          <t>Denny Sanjaya</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>85813046313</t>
+          <t>87880208886</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Jl. Gatot Subroto No. A1-A2 RT.001/RW.4, Sangiang Jaya, Kec. Periuk, Kota Tangerang, Banten 15134</t>
+          <t>Jl. Raya Villa Tangerang Indah RT.003/RW.012 Gebang Raya Kec. Periuk Tangerang 15132</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -4875,17 +4875,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>E684</t>
+          <t>E150</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO SANGIANG TANGERANG</t>
+          <t>ERAFONE CILEGON CENTER MALL</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>CILEGON</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -4895,17 +4895,17 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Denny Sanjaya</t>
+          <t>Arif Abdurahman Aziz</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>87880208886</t>
+          <t>81287922331</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Villa Tangerang Indah RT.003/RW.012 Gebang Raya Kec. Periuk Tangerang 15132</t>
+          <t>Cilegon Center Mall Lt 1 No. 14 , Jl. Ahmad Yani No. 11 Sukmajaya, Kec. Jombang, Kota Cilegon, Banten 42416</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -4920,17 +4920,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>E150</t>
+          <t>E081</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE CILEGON CENTER MALL</t>
+          <t>ERAFONE MALL OF SERANG</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>CILEGON</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4940,17 +4940,17 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Arif Abdurahman Aziz</t>
+          <t>Andi Saputra</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>81287922331</t>
+          <t>87875027979</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Cilegon Center Mall Lt 1 No. 14 , Jl. Ahmad Yani No. 11 Sukmajaya, Kec. Jombang, Kota Cilegon, Banten 42416</t>
+          <t>Mall of Serang Lantai 1 No. 20, Jl. Akses Tol Serang Tim., Panancangan, Kec. Cipocok Jaya, Kota Serang, Banten 42124</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
@@ -4965,12 +4965,12 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>E081</t>
+          <t>E209</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MALL OF SERANG</t>
+          <t>ERAFONE RUKO AHMAD YANI SERANG</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -4985,17 +4985,17 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Andi Saputra</t>
+          <t>Depih Harlan</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>87875027979</t>
+          <t>87701418112</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Mall of Serang Lantai 1 No. 20, Jl. Akses Tol Serang Tim., Panancangan, Kec. Cipocok Jaya, Kota Serang, Banten 42124</t>
+          <t>Jl. Jendral Ahmad Yani No.104 RT RW 001/002 Sumurpecung, Kec. Serang, Kota Serang, Banten 42117</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -5010,17 +5010,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>E209</t>
+          <t>E194</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO AHMAD YANI SERANG</t>
+          <t>ERAFONE RUKO RANGKASBITUNG</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>RANGKASBITUNG</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -5030,17 +5030,17 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Depih Harlan</t>
+          <t>Fardan Ega Pirmansyah</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>83866359264</t>
+          <t>85694929109</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Jl. Jendral Ahmad Yani No.104 RT RW 001/002 Sumurpecung, Kec. Serang, Kota Serang, Banten 42117</t>
+          <t>Ruko Multatuli Rangkas Bitung, Jl. Multatuli No.95, Muara Ciujung Bar., Kec. Rangkasbitung, Kabupaten Lebak, Banten 42312</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -5055,17 +5055,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>E194</t>
+          <t>E308</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO RANGKASBITUNG</t>
+          <t>ERAFONE RUKO MAYOR SAFEI SERANG</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>RANGKASBITUNG</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -5075,17 +5075,17 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Fardan Ega Pirmansyah</t>
+          <t>Wita Gita Widianti</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>85694929109</t>
+          <t>87786221611</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Ruko Multatuli Rangkas Bitung, Jl. Multatuli No.95, Muara Ciujung Bar., Kec. Rangkasbitung, Kabupaten Lebak, Banten 42312</t>
+          <t>Jalan Mayor Safei Serang , Kel Lontarbaru , Kec Serang , Kota Serang Banten Kode POS 42115</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -5100,17 +5100,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>E308</t>
+          <t>E320</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO MAYOR SAFEI SERANG</t>
+          <t>ERAFONE RUKO PANDEGLANG BANTEN</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>PANDEGLANG</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -5120,17 +5120,17 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Tubagus Hanifan</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>85921222664</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Jalan Mayor Safei Serang , Kel Lontarbaru , Kec Serang , Kota Serang Banten Kode POS 42115</t>
+          <t>Jl. Serang Pandeglang, Kel. Pandeglang Kec. Pandeglang, Kab. Pandeglang, Banten kode Pos 42211</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -5145,12 +5145,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>E320</t>
+          <t>E589</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO PANDEGLANG BANTEN</t>
+          <t>ERAFONE RUKO PANIMBANG PANDEGLANG</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -5165,17 +5165,17 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>TB.HANIFAN</t>
+          <t>Ahmad Hidayatulloh</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>85921222664</t>
+          <t>85778211772</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Jl. Serang Pandeglang, Kel. Pandeglang Kec. Pandeglang, Kab. Pandeglang, Banten kode Pos 42211</t>
+          <t>JL. Raya Tanjung - Panimbang, Kp. Padahayu RT 01/04 Ds. Panimbang jaya, Kec. Panimbang Kab. Pandeglang 42281</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>E589</t>
+          <t>E499</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO PANIMBANG PANDEGLANG</t>
+          <t>ERAFONE LABUAN PANDEGLANG</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -5210,17 +5210,17 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Arby Rabiul Tsani</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87778810806</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>JL. Raya Tanjung - Panimbang, Kp. Padahayu RT 01/04 Ds. Panimbang jaya, Kec. Panimbang Kab. Pandeglang 42281</t>
+          <t>Jl. Jend. Sudirman No. 99, Muncang Labuan, Kec. Labuang, Pandeglang, Banten 42264</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -5235,17 +5235,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>E499</t>
+          <t>E544</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE LABUAN PANDEGLANG</t>
+          <t>ERAFONE RUKO MULTIBRAND CILEGON</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>PANDEGLANG</t>
+          <t>CILEGON</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5255,17 +5255,17 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ahmad Khusnul</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>895336274142</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Jl. Jend. Sudirman No. 99, Muncang Labuan, Kec. Labuang, Pandeglang, Banten 42264</t>
+          <t>Jl. Simpang Tiga No.13 RT.06 RW.01 Kel. Ramanuju Kec. Purwakarta Cilegon, Banten 42411</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
@@ -5280,17 +5280,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>E544</t>
+          <t>E821</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO MULTIBRAND CILEGON</t>
+          <t>ERAFONE MB ANYER</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>CILEGON</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5300,17 +5300,17 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Ahmad Khusnul</t>
+          <t>Ali Rohman</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>895336274142</t>
+          <t>82249001138</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Jl. Simpang Tiga No.13 RT.06 RW.01 Kel. Ramanuju Kec. Purwakarta Cilegon, Banten 42411</t>
+          <t>Jalan Raya Anyer Sirih Kec Anyer Kabupaten Serang Banten 42166</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -5325,12 +5325,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>E821</t>
+          <t>E822</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB ANYER</t>
+          <t>ERAFONE MB KRAGILAN</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -5345,17 +5345,17 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Marvel Ficky Watuseke</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>0254-7960524</t>
+          <t>81514421196</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Jalan Raya Anyer Sirih Kec Anyer Kabupaten Serang Banten 42166</t>
+          <t>Jalan raya serang- KM 15, Kragilan, kec Kragilan,Kab Serang BANTEN 42184</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
@@ -5370,37 +5370,37 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>E822</t>
+          <t>E833</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB KRAGILAN</t>
+          <t>ERAFONE RANGKASBITUNG 2</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>RANGKASBITUNG</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>M Dede Nurjeli</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>0254-7901771</t>
+          <t>85894631045</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Jalan raya serang- KM 15, Kragilan, kec Kragilan,Kab Serang BANTEN 42184</t>
+          <t>JL. Sunan kalijaga No.325 Kp. Papanggo RT.01 RW.02 Kel. Cijoro Pasir Rangkasbitung</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
@@ -5415,37 +5415,37 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>E833</t>
+          <t>E879</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RANGKASBITUNG 2</t>
+          <t>ERAFONE MB CIPARE</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>RANGKASBITUNG</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Hendro Wijaya</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81906450517</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>JL. Sunan kalijaga No.325 Kp. Papanggo RT.01 RW.02 Kel. Cijoro Pasir Rangkasbitung</t>
+          <t>JL. Raya Pandeglang Sempu, Banten Girang RT.001 RW.017 Kel. Cipare Kec. Serang Kota Serang Banten</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -5460,37 +5460,37 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>E879</t>
+          <t>M027</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB CIPARE</t>
+          <t>ERAFONE AND MORE CIPUTAT</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Mochamad Helmi Alatas</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>0254-4078399</t>
+          <t>85155303034</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>JL. Raya Pandeglang Sempu, Banten Girang RT.001 RW.017 Kel. Cipare Kec. Serang Kota Serang Banten</t>
+          <t>Jl. Dewi Sartika No.12 D, Cipayung, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -5505,12 +5505,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>M027</t>
+          <t>E191</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE CIPUTAT</t>
+          <t>ERAFONE RUKO SURYA KENCANA PAMULANG</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5520,22 +5520,22 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>Mochamad Helmi Alatas</t>
+          <t>Muhammad Sidik</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>85117769126</t>
+          <t>85770795112</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Jl. Dewi Sartika No.12 D, Cipayung, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
+          <t>Jl. Surya Kencana No.60, Pamulang Bar., Kec. Pamulang, Kota Tangerang Selatan, Banten 15417</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
@@ -5550,12 +5550,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>E191</t>
+          <t>F022</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO SURYA KENCANA PAMULANG</t>
+          <t>ERAFONE 2.5 PAMULANG</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5570,17 +5570,17 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Untung</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>87777192252</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Jl. Surya Kencana No.60, Pamulang Bar., Kec. Pamulang, Kota Tangerang Selatan, Banten 15417</t>
+          <t>Jalan siliwangi no. 2 pondok benda, kec. Pamulang, Banten 15417</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -5595,12 +5595,12 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>F022</t>
+          <t>E484</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 PAMULANG</t>
+          <t>ERAFONE SERPONG PARADISE WALK</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -5615,17 +5615,17 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Angga Ardian Saputra</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89608218065</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Jalan siliwangi no. 2 pondok benda, kec. Pamulang, Banten 15417</t>
+          <t>Jalan Graha Raya Boulevard, Paku Jaya, Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -5640,17 +5640,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>E484</t>
+          <t>E087</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE SERPONG PARADISE WALK</t>
+          <t>ERAFONE ITC BSD</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5660,17 +5660,17 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Aan</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81990000098</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Jalan Graha Raya Boulevard, Paku Jaya, Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
+          <t>BSD City, ITC BSD Lantai 3 D3A-6, Jl. Pahlawan Seribu, Lengkong Wetan, Tangerang, Kota Tangerang Selatan, Banten 15321</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -5685,17 +5685,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>E087</t>
+          <t>E941</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE ITC BSD</t>
+          <t>ERAFONE MB RAYA SERPONG</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -5705,17 +5705,17 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ari Firdaus Saputra</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>021-5381354</t>
+          <t>85718574849</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>BSD City, ITC BSD Lantai 3 D3A-6, Jl. Pahlawan Seribu, Lengkong Wetan, Tangerang, Kota Tangerang Selatan, Banten 15321</t>
+          <t>Jalan Benda Permai Raya B8/8-B8/9, RT 001, RW 010,Kel/Desa Pondok Benda, Kecamatan Pamulang, Kota Tangerang Selatan, Provinsi Banten</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -5730,12 +5730,12 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>E941</t>
+          <t>E586</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB RAYA SERPONG</t>
+          <t>ERAFONE RUKO GRAHA RAYA</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5750,17 +5750,17 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A Rahman</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>895326032806</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Jalan Benda Permai Raya B8/8-B8/9, RT 001, RW 010,Kel/Desa Pondok Benda, Kecamatan Pamulang, Kota Tangerang Selatan, Provinsi Banten</t>
+          <t>Jl. Boulevard Graha Raya NO.B15, Paku Jaya, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -5775,12 +5775,12 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>E586</t>
+          <t>E834</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO GRAHA RAYA</t>
+          <t>ERAFONE KEDAUNG TANGSEL</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5790,22 +5790,22 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Samsuri</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>82213538214</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Jl. Boulevard Graha Raya NO.B15, Paku Jaya, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
+          <t>Jl. Pondok Cabe Raya No.9, Kec. Pamulang, Kota Tangerang Selatan, Banten 15418</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -5820,37 +5820,37 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>E834</t>
+          <t>E082</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE KEDAUNG TANGSEL</t>
+          <t>ERAFONE LIVING WORLD ALAM SUTERA</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Indra Setiawan</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81519578723</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Jl. Pondok Cabe Raya No.9, Kec. Pamulang, Kota Tangerang Selatan, Banten 15418</t>
+          <t>Living World Alam Sutera 1st floor No.30B Jalan Alam Sutera Boulevard Kav. 21, Pakulonan, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15325</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
@@ -5865,12 +5865,12 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>E082</t>
+          <t>E088</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE LIVING WORLD ALAM SUTERA</t>
+          <t>ERAFONE AEON MAL BSD CITY</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -5885,65 +5885,20 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Indra Setiawan</t>
+          <t>Gina Tania</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>81519578723</t>
+          <t>85880148262</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Living World Alam Sutera 1st floor No.30B Jalan Alam Sutera Boulevard Kav. 21, Pakulonan, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15325</t>
+          <t>AEON Mal BSD City Lantai 3 LOT 3-15 Jl. Grand Boulevard BSD City Pagedangan, Kec. Pagedangan, Tangerang, Banten 15345</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
-        <is>
-          <t>Aktif</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="n">
-        <v>121</v>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>E088</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>ERAFONE AEON MAL BSD CITY</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>TANGERANG</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>Erafone Multibrand</t>
-        </is>
-      </c>
-      <c r="F122" s="2" t="inlineStr">
-        <is>
-          <t>Gina Tania</t>
-        </is>
-      </c>
-      <c r="G122" s="2" t="inlineStr">
-        <is>
-          <t>85880148262</t>
-        </is>
-      </c>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t>AEON Mal BSD City Lantai 3 LOT 3-15 Jl. Grand Boulevard BSD City Pagedangan, Kec. Pagedangan, Tangerang, Banten 15345</t>
-        </is>
-      </c>
-      <c r="I122" s="2" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>

</xml_diff>

<commit_message>
Remove closed store E620 (Erafone 2.5 Pajajaran Pamulang)
Store has closed, so it no longer belongs in the active Erafone
Region 5 store list. 119 stores remain.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ERAFONE-STORE-LIST-SEPTEMBER-2026.xlsx
+++ b/ERAFONE-STORE-LIST-SEPTEMBER-2026.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2940,12 +2940,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>E620</t>
+          <t>M104</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 PAJAJARAN PAMULANG</t>
+          <t>MEGASTORE RUKO REMPOA CIPUTAT</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2955,22 +2955,22 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Heru Bachtiar</t>
+          <t>Iqbal Firdaus</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>83811921019</t>
+          <t>85959388797</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Jl. Pajajaran No.39, Pamulang Barat Kec. Pamulang Tangerang Selatan</t>
+          <t>Jl. Pahlawan No.02 RT.5/RW.3 kelurahan;Rempoa Kecamatan; Ciputat Timur</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -2985,12 +2985,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>M104</t>
+          <t>E321</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO REMPOA CIPUTAT</t>
+          <t>ERAFONE RUKO SUDIMARA CIPUTAT</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -3000,22 +3000,22 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Iqbal Firdaus</t>
+          <t>Muhamad Igfir Refi Syarip</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>85959388797</t>
+          <t>895395257767</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Jl. Pahlawan No.02 RT.5/RW.3 kelurahan;Rempoa Kecamatan; Ciputat Timur</t>
+          <t>Jl. Jombang Raya No 21 RT/RW 02/02 Kelurahan Jombang, kecamatan Ciputat, Kota Tangerang Selatan, Banten 15414</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3030,12 +3030,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>E321</t>
+          <t>E704</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO SUDIMARA CIPUTAT</t>
+          <t>ERAFONE RUKO DEWANTARA CIPUTAT</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3050,17 +3050,17 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Muhamad Igfir Refi Syarip</t>
+          <t>Muhammad Riduan Wahid</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>895395257767</t>
+          <t>89603352071</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Jl. Jombang Raya No 21 RT/RW 02/02 Kelurahan Jombang, kecamatan Ciputat, Kota Tangerang Selatan, Banten 15414</t>
+          <t>Jl. Ki Hajar Dewantara No.22, RT.1/RW.3, Ciputat, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3075,12 +3075,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>E704</t>
+          <t>E043</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO DEWANTARA CIPUTAT</t>
+          <t>ERAFONE PLAZA BINTARO JAYA</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -3095,17 +3095,17 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Riduan Wahid</t>
+          <t>Serpon</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>89603352071</t>
+          <t>81291059132</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Jl. Ki Hajar Dewantara No.22, RT.1/RW.3, Ciputat, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
+          <t>Plaza Bintaro Jaya Lantai 1 No. 12A Jl. Bintaro Utama Sektor 3-A, Pd. Karya, Pd. Aren, Kota Tangerang Selatan, Banten 15225</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>E043</t>
+          <t>E685</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE PLAZA BINTARO JAYA</t>
+          <t>ERAFONE MB PONDOK BETUNG</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3140,17 +3140,17 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Serpon</t>
+          <t>Rizki Tazakka</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>81291059132</t>
+          <t>81779941945</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Plaza Bintaro Jaya Lantai 1 No. 12A Jl. Bintaro Utama Sektor 3-A, Pd. Karya, Pd. Aren, Kota Tangerang Selatan, Banten 15225</t>
+          <t>Jl. Ceger Raya No. 22 B , Kel. Pondok karya Kec. Pondok Aren , Kota Tangerang Selatan , Banten 15225</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -3165,12 +3165,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>E685</t>
+          <t>E391</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB PONDOK BETUNG</t>
+          <t>ERAFONE RUKO WR SUPRATMAN CIPUTAT</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -3185,17 +3185,17 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Rizki Tazakka</t>
+          <t>Heru Bachtiar</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>81779941945</t>
+          <t>83811921019</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Jl. Ceger Raya No. 22 B , Kel. Pondok karya Kec. Pondok Aren , Kota Tangerang Selatan , Banten 15225</t>
+          <t>Jl. WR Supratman No 124 kecamatan. Kecamatan Ciputat Timur. keluraha Cempaka Putih. Banten 15412</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -3210,17 +3210,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>E391</t>
+          <t>E084</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO WR SUPRATMAN CIPUTAT</t>
+          <t>ERAFONE 1 SUPERMALL KARAWACI</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3230,17 +3230,17 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Heru Bachtiar</t>
+          <t>Alfian</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>83811921019</t>
+          <t>85747292806</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Jl. WR Supratman No 124 kecamatan. Kecamatan Ciputat Timur. keluraha Cempaka Putih. Banten 15412</t>
+          <t>Supermall Karawaci Lantai LG No.3A-6A E-CENTER, Jl. Boulevard Diponegoro No.105, Bencongan, Kec. Klp. Dua, Kota Tangerang, Banten 15811</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -3255,37 +3255,37 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>E084</t>
+          <t>M163</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 1 SUPERMALL KARAWACI</t>
+          <t>ERAFONE AND MORE SERPONG</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Alfian</t>
+          <t>Mochammad Ramdan Akbar</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>85747292806</t>
+          <t>85894568558</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Supermall Karawaci Lantai LG No.3A-6A E-CENTER, Jl. Boulevard Diponegoro No.105, Bencongan, Kec. Klp. Dua, Kota Tangerang, Banten 15811</t>
+          <t>Jl. MH. Thamrin No.7, Pakualam, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15143</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -3300,37 +3300,37 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>M163</t>
+          <t>E777</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE SERPONG</t>
+          <t>ERAFONE MB CIHUNI PAGEDANGAN (ERAFONE CIHUNI GADING SERPONG)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Mochammad Ramdan Akbar</t>
+          <t>Mulyana</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>85894568558</t>
+          <t>87776764678</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Jl. MH. Thamrin No.7, Pakualam, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15143</t>
+          <t>ruko North sorrento square No.1 Jl.Ir sukarno cihuni,kec pagedangan,kabupaten Tangerang ,Banten 15332</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3345,12 +3345,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>E777</t>
+          <t>E873</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB CIHUNI PAGEDANGAN (ERAFONE CIHUNI GADING SERPONG)</t>
+          <t>ERAFONE MB LEGOK</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -3365,17 +3365,17 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Mulyana</t>
+          <t>Andri Sundara</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>87776764678</t>
+          <t>81318321003</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>ruko North sorrento square No.1 Jl.Ir sukarno cihuni,kec pagedangan,kabupaten Tangerang ,Banten 15332</t>
+          <t>Jln. Raya PLP Curug No. 95 Kec. Legok, Kab. Tangerang Banten 15820</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -3390,12 +3390,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>E873</t>
+          <t>E874</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB LEGOK</t>
+          <t>ERAFONE MULTIBRAND DASANA INDAH</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -3410,17 +3410,17 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Andri Sundara</t>
+          <t>Rezky Nabila</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>81318321003</t>
+          <t>89678086600</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Jln. Raya PLP Curug No. 95 Kec. Legok, Kab. Tangerang Banten 15820</t>
+          <t>Jln. Raya Dasana Indah Blok SA1 No. 11, Bojong Nangka, Kec. Kelapa Dua Tangerang, Banten 15810</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3435,12 +3435,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>E874</t>
+          <t>E813</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MULTIBRAND DASANA INDAH</t>
+          <t>ERAFONE MULTIBRAND SERPONG GARDEN CISAUK</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -3455,17 +3455,17 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Rezky Nabila</t>
+          <t>Diki Febriyanto</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>89678086600</t>
+          <t>895363851554</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Jln. Raya Dasana Indah Blok SA1 No. 11, Bojong Nangka, Kec. Kelapa Dua Tangerang, Banten 15810</t>
+          <t>Jl. Raya Cisauk Lapan Jl. Ruko Serpong Garden ruko 3 No.21, Cibogo, Kec. Cisauk, Kabupaten Tangerang, Banten 15341</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3480,12 +3480,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>E813</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MULTIBRAND SERPONG GARDEN CISAUK</t>
+          <t>MEGASTORE SUMMARECON MAL SERPONG</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -3495,22 +3495,22 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Diki Febriyanto</t>
+          <t>Niko</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>895363851554</t>
+          <t>87771807710</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Cisauk Lapan Jl. Ruko Serpong Garden ruko 3 No.21, Cibogo, Kec. Cisauk, Kabupaten Tangerang, Banten 15341</t>
+          <t>Summarecon Mall Serpong Lantai 2F No. 17A, Jalan Gading Serpong Boulevard No.1, No.2 F, Pakulonan Bar., Kec. Klp. Dua, Tangerang, Banten 15810</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -3525,12 +3525,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>M019</t>
+          <t>M013</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE SUMMARECON MAL SERPONG</t>
+          <t>MEGASTORE SUPERMAL KARAWACI</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -3545,17 +3545,17 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Niko</t>
+          <t>Rudi Herdiyanto</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>87771807710</t>
+          <t>87770836816</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Summarecon Mall Serpong Lantai 2F No. 17A, Jalan Gading Serpong Boulevard No.1, No.2 F, Pakulonan Bar., Kec. Klp. Dua, Tangerang, Banten 15810</t>
+          <t>Supermal Karawaci Lantai 1 Unit FF 51-52 105. Jl. Boulevard Diponegoro No.105, Bencongan, Kec. Klp. Dua, Kota Tangerang, Banten 15811</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>M013</t>
+          <t>M222</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE SUPERMAL KARAWACI</t>
+          <t>ERAFONE AND MORE EASTVARA MALL</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -3585,22 +3585,22 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Rudi Herdiyanto</t>
+          <t>Reno Dharmawan</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>87770836816</t>
+          <t>87808367901</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Supermal Karawaci Lantai 1 Unit FF 51-52 105. Jl. Boulevard Diponegoro No.105, Bencongan, Kec. Klp. Dua, Kota Tangerang, Banten 15811</t>
+          <t>Eastvara Mall, Jl. BSD Boulevard Utara, Cijantra, Kec. Pagedangan, Kabupaten Tangerang, Banten 15854</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -3615,12 +3615,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>M222</t>
+          <t>E369</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE EASTVARA MALL</t>
+          <t>ERAFONE FRANCHISE RUKO BOROBUDUR RAYA</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3630,22 +3630,22 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Reno Dharmawan</t>
+          <t>Ramdani Andika Pramandana</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>87808367901</t>
+          <t>82221833394</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Eastvara Mall, Jl. BSD Boulevard Utara, Cijantra, Kec. Pagedangan, Kabupaten Tangerang, Banten 15854</t>
+          <t>Jl. Borobudur Raya Kel, Cibodas Baru, Kec.Cibodas Kota Tangerang</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -3660,12 +3660,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>E369</t>
+          <t>E370</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE FRANCHISE RUKO BOROBUDUR RAYA</t>
+          <t>ERAFONE FRANCHISE RUKO BERINGIN KARAWACI</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3680,17 +3680,17 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Ramdani Andika Pramandana</t>
+          <t>Sugianto</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>82221833394</t>
+          <t>85888026212</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Jl. Borobudur Raya Kel, Cibodas Baru, Kec.Cibodas Kota Tangerang</t>
+          <t>Jl. Beringin Raya Kel. Nusa Jaya, Kec. Tangerang Kota Tangerang</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -3705,12 +3705,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>E370</t>
+          <t>E221</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE FRANCHISE RUKO BERINGIN KARAWACI</t>
+          <t>ERAFONE AND MORE CIPUTRA CITRARAYA TANGERANG</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3720,22 +3720,22 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Sugianto</t>
+          <t>Elvirawati</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>85888026212</t>
+          <t>87880648402</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Jl. Beringin Raya Kel. Nusa Jaya, Kec. Tangerang Kota Tangerang</t>
+          <t>Jl. Citra Raya Boulevard No.38 Mall Citra Lt. 2 unit C 19-12, Ciakar, Kec. Panongan, Kabupaten Tangerang, Banten 15710</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -3750,12 +3750,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>E221</t>
+          <t>F058</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE CIPUTRA CITRARAYA TANGERANG</t>
+          <t>ERAFONE 2.5 TELAGA BESTARI</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3765,22 +3765,22 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Elvirawati</t>
+          <t>Aditya Anjasmara</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>87880648402</t>
+          <t>87778274871</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Jl. Citra Raya Boulevard No.38 Mall Citra Lt. 2 unit C 19-12, Ciakar, Kec. Panongan, Kabupaten Tangerang, Banten 15710</t>
+          <t>Jl. Taman Palem Raya No.12, Wana Kerta, kec sindang jaya1, Kabupaten Tangerang, Banten 15560</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -3795,12 +3795,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>F058</t>
+          <t>M048</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 TELAGA BESTARI</t>
+          <t>MEGASTORE RUKO CIKUPA</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3810,22 +3810,22 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Aditya Anjasmara</t>
+          <t>Dede Dermawan</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>87778274871</t>
+          <t>85285954784</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Jl. Taman Palem Raya No.12, Wana Kerta, kec sindang jaya1, Kabupaten Tangerang, Banten 15560</t>
+          <t>Ruko Cikupa, Jl. Raya Serang Balaraja, Sukanagara, Kec. Cikupa, Tangerang, Banten 15710</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -3840,12 +3840,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>M048</t>
+          <t>M167</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO CIKUPA</t>
+          <t>ERAFONE AND MORE TELUK NAGA</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3855,22 +3855,22 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Dede Dermawan</t>
+          <t>Jatonggo Silitonga</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>85285954784</t>
+          <t>85782286690</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Ruko Cikupa, Jl. Raya Serang Balaraja, Sukanagara, Kec. Cikupa, Tangerang, Banten 15710</t>
+          <t>Kampung Melayu Barat RT 01/RW 02 No. II-C, Kp. Melayu Barat, Kec. Teluknaga, Tangerang Kabupaten, Banten 15510</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -3885,12 +3885,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>M167</t>
+          <t>E627</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE TELUK NAGA</t>
+          <t>ERAFONE RUKO CISOKA</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3900,22 +3900,22 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Jatonggo Silitonga</t>
+          <t>Fahrul Yanuar</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>85782286690</t>
+          <t>8985500577</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Kampung Melayu Barat RT 01/RW 02 No. II-C, Kp. Melayu Barat, Kec. Teluknaga, Tangerang Kabupaten, Banten 15510</t>
+          <t>Jl. Raya Cisoka Adiyasa No .35-36 Rt 001/Rw/001 Kp Lukun Sukatani ,Kec Cisoka Kabupaten Tangerang Banten</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -3930,12 +3930,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>E627</t>
+          <t>E253</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO CISOKA</t>
+          <t>ERAFONE RUKO CURUG TANGERANG</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3950,17 +3950,17 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Fahrul Yanuar</t>
+          <t>Teguh Prakoso</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>8985500577</t>
+          <t>81287162443</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Cisoka Adiyasa No .35-36 Rt 001/Rw/001 Kp Lukun Sukatani ,Kec Cisoka Kabupaten Tangerang Banten</t>
+          <t>Jl. Raya PLP Curug No.16, Suka Bakti, Kec. Curug, Tangerang, Banten 15810</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3975,12 +3975,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>E253</t>
+          <t>E787</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO CURUG TANGERANG</t>
+          <t>ERAFONE MB TIGARAKSA</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3995,17 +3995,17 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Teguh Prakoso</t>
+          <t>Nana Pratama</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>81287162443</t>
+          <t>85711100857</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya PLP Curug No.16, Suka Bakti, Kec. Curug, Tangerang, Banten 15810</t>
+          <t>JL. Syeh Mubarok Matagara No.9 RT 001/004, TIGARAKSA TANGERANG Banten 15720</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>E787</t>
+          <t>E848</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB TIGARAKSA</t>
+          <t>ERAFONE PASAR KEMIS</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4040,17 +4040,17 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Nana Pratama</t>
+          <t>Irfan Supiandi</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>85711100857</t>
+          <t>81276004200</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>JL. Syeh Mubarok Matagara No.9 RT 001/004, TIGARAKSA TANGERANG Banten 15720</t>
+          <t>JL.Taman Sukamatri Raya A/12 Kel Sukamatri Kec. Pasar Kemis Kab.Tangerang 15560 Banten</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -4065,12 +4065,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>E848</t>
+          <t>E812</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE PASAR KEMIS</t>
+          <t>ERAFONE RUKO KUTABUMI</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -4085,17 +4085,17 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Irfan Supiandi</t>
+          <t>Edi Suryadi</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>81276004200</t>
+          <t>85959594176</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>JL.Taman Sukamatri Raya A/12 Kel Sukamatri Kec. Pasar Kemis Kab.Tangerang 15560 Banten</t>
+          <t>Jl. Raya Regency II Kel. Kuta Jaya Kec. Ps. Kemis Kab. Tangerang 15560</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -4110,12 +4110,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>E812</t>
+          <t>E201</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO KUTABUMI</t>
+          <t>ERAFONE RUKO KRESEK BALARAJA</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4130,17 +4130,17 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Edi Suryadi</t>
+          <t>Mochamad Ryan Krisdiana</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>85959594176</t>
+          <t>81315592228</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Regency II Kel. Kuta Jaya Kec. Ps. Kemis Kab. Tangerang 15560</t>
+          <t>Jl. Raya Kresek, Saga, Kec. Balaraja, Tangerang, Banten 15610</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4155,12 +4155,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>E201</t>
+          <t>E744</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO KRESEK BALARAJA</t>
+          <t>ERAFONE RUKO RAJEG TANGERANG</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -4175,17 +4175,17 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Mochamad Ryan Krisdiana</t>
+          <t>Misbahul Badri</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>81315592228</t>
+          <t>81283260410</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Kresek, Saga, Kec. Balaraja, Tangerang, Banten 15610</t>
+          <t>Jl. Raya Ps. Kemis, Mekarsari Kel. Mekarsari Kec. Rajeg Kab. Tangerang Banten 15540.</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -4200,12 +4200,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>E744</t>
+          <t>F066</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO RAJEG TANGERANG</t>
+          <t>ERAFONE 2.5 SEPATAN</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -4215,22 +4215,22 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Misbahul Badri</t>
+          <t>Ade Rizky Pajarian</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>81283260410</t>
+          <t>81574755707</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Ps. Kemis, Mekarsari Kel. Mekarsari Kec. Rajeg Kab. Tangerang Banten 15540.</t>
+          <t>Jl. Raya Mauk Jl. Tangerang Golden City No.3</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -4245,17 +4245,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>F066</t>
+          <t>F079</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 SEPATAN</t>
+          <t>ERAFONE 2.5 GRAND BATAVIA</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>KABUPATEN TANGERANG</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -4265,17 +4265,17 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Ade Rizky Pajarian</t>
+          <t>Oktavian Nurrahmat</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>81574755707</t>
+          <t>85932222992</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Mauk Jl. Tangerang Golden City No.3</t>
+          <t>Jalan Raya Grand Batavia RT02/RW019 Kel.Sindangsari Kec.Pasar Kemis Kab.Tangerang,Banten 15560</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
@@ -4290,37 +4290,37 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>F079</t>
+          <t>M021</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 GRAND BATAVIA</t>
+          <t>MEGASTORE RUKO CILEDUG</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>KABUPATEN TANGERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Oktavian Nurrahmat</t>
+          <t>Fahruk Azhara</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>85932222992</t>
+          <t>85822017978</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Jalan Raya Grand Batavia RT02/RW019 Kel.Sindangsari Kec.Pasar Kemis Kab.Tangerang,Banten 15560</t>
+          <t>Jl. Ciledug Raya No. 30 RT.006/RW.002, Petukangan Utara, Kec. Pesanggrahan, Kota Tangerang, Banten 15156</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -4335,37 +4335,37 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>M021</t>
+          <t>E231</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO CILEDUG</t>
+          <t>ERAFONE RUKO COKROAMINOTO CILEDUG</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Fahruk Azhara</t>
+          <t>Muhammad Dendy</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>85822017978</t>
+          <t>81281736135</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Jl. Ciledug Raya No. 30 RT.006/RW.002, Petukangan Utara, Kec. Pesanggrahan, Kota Tangerang, Banten 15156</t>
+          <t>Jln. HOS Cokroaminoto No. 29 RT. 002 RW. 004, Karang Timur, Karang Tengah, Ciledug, Tangerang</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>E231</t>
+          <t>F003</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO COKROAMINOTO CILEDUG</t>
+          <t>Erafone Ciledug 2.5 Raya</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -4400,17 +4400,17 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Dendy</t>
+          <t>Mahfudin</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>81281736135</t>
+          <t>816652158</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Jln. HOS Cokroaminoto No. 29 RT. 002 RW. 004, Karang Timur, Karang Tengah, Ciledug, Tangerang</t>
+          <t>Jl Ciledug Raya No 9 RT/RW 001/009, Larangan Indah, Kec Larangan, Kota Tangerang Banten 15154</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -4425,12 +4425,12 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>F003</t>
+          <t>M093</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Erafone Ciledug 2.5 Raya</t>
+          <t>MEGASTORE RUKO CIPONDOH TANGERANG</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -4440,22 +4440,22 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Mahfudin</t>
+          <t>Cukat Yoga Aditya</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>816652158</t>
+          <t>89526719552</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Jl Ciledug Raya No 9 RT/RW 001/009, Larangan Indah, Kec Larangan, Kota Tangerang Banten 15154</t>
+          <t>Jl KH Hasyim Asyhari RT003/RW003 No. 67B Cipondoh Tangerang</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -4470,12 +4470,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>M093</t>
+          <t>E290</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO CIPONDOH TANGERANG</t>
+          <t>ERAFONE FRANCHISE RUKO PORIS</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4485,22 +4485,22 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Cukat Yoga Aditya</t>
+          <t>Hasril Oktama</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>89526719552</t>
+          <t>8976118817</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Jl KH Hasyim Asyhari RT003/RW003 No. 67B Cipondoh Tangerang</t>
+          <t>Jalan Poris indah Raya, Ruko Paradise Eksklusif. Poris Gaga Batu Ceper Tangerang</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -4515,12 +4515,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>E290</t>
+          <t>E646</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE FRANCHISE RUKO PORIS</t>
+          <t>ERAFONE BATU CEPER</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4530,22 +4530,22 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Hasril Oktama</t>
+          <t>Saiful Zuhdi</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>8976118817</t>
+          <t>81284458691</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Jalan Poris indah Raya, Ruko Paradise Eksklusif. Poris Gaga Batu Ceper Tangerang</t>
+          <t>Jl. Halim Perdana Kusuma, RT.002/RW.001, Jurumudi Baru, Kec. Batuceper, Kota Tangerang, Banten 15122</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>E646</t>
+          <t>E119</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE BATU CEPER</t>
+          <t>ERAFONE TANGERANG CITY MALL</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Saiful Zuhdi</t>
+          <t>Mega Nurhatifah, SE</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>81284458691</t>
+          <t>81284456745</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Jl. Halim Perdana Kusuma, RT.002/RW.001, Jurumudi Baru, Kec. Batuceper, Kota Tangerang, Banten 15122</t>
+          <t>Tangerang City Mall Lantai LG, Jl. Jenderal Sudirman No.1, RT.001/RW.005, Babakan, Kec. Tangerang, Kota Tangerang, Banten 15117</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -4605,12 +4605,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>E119</t>
+          <t>E696</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE TANGERANG CITY MALL</t>
+          <t>ERAFONE MB RASUNA SAID</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4620,22 +4620,22 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Mega Nurhatifah, SE</t>
+          <t>Muhamad Riyanto</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>81284456745</t>
+          <t>87817170393</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Tangerang City Mall Lantai LG, Jl. Jenderal Sudirman No.1, RT.001/RW.005, Babakan, Kec. Tangerang, Kota Tangerang, Banten 15117</t>
+          <t>JL.HR Rasuna Said RT01/RW 02 Pakojan, kec.Pinang, Kota Tangerang, Banten 15142</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -4650,12 +4650,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>E696</t>
+          <t>M176</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB RASUNA SAID</t>
+          <t>ERAFONE AND MORE KISAMAUN</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4665,22 +4665,22 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Muhamad Riyanto</t>
+          <t>Muammar Alfis</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>87817170393</t>
+          <t>81212400080</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>JL.HR Rasuna Said RT01/RW 02 Pakojan, kec.Pinang, Kota Tangerang, Banten 15142</t>
+          <t>Jl Kisamaun No 89G RT/RW 002/007 Kel. Sukasari Kec. Tangerang Kota Tangerang</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -4695,12 +4695,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>M176</t>
+          <t>E422</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE KISAMAUN</t>
+          <t>ERAFONE RUKO M TOHA TANGERANG</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -4710,22 +4710,22 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Muammar Alfis</t>
+          <t>Michael Roma Nelson</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>81212400080</t>
+          <t>81212456692</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Jl Kisamaun No 89G RT/RW 002/007 Kel. Sukasari Kec. Tangerang Kota Tangerang</t>
+          <t>Jl. Moh. Toha. RT 001/Rw.008 Pabuaran Tumpeng, Kec Karawaci, Kota Tangerang, 15114</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
@@ -4740,12 +4740,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>E422</t>
+          <t>M061</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO M TOHA TANGERANG</t>
+          <t>MEGASTORE RUKO JATIUWUNG</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -4755,22 +4755,22 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Megastore</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Michael Roma Nelson</t>
+          <t>Santo</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>81212456692</t>
+          <t>85813046313</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Jl. Moh. Toha. RT 001/Rw.008 Pabuaran Tumpeng, Kec Karawaci, Kota Tangerang, 15114</t>
+          <t>Jl. Gatot Subroto No. A1-A2 RT.001/RW.4, Sangiang Jaya, Kec. Periuk, Kota Tangerang, Banten 15134</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -4785,12 +4785,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>M061</t>
+          <t>E684</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>MEGASTORE RUKO JATIUWUNG</t>
+          <t>ERAFONE RUKO SANGIANG TANGERANG</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4800,22 +4800,22 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Erafone Megastore</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Santo</t>
+          <t>Denny Sanjaya</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>85813046313</t>
+          <t>87880208886</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Jl. Gatot Subroto No. A1-A2 RT.001/RW.4, Sangiang Jaya, Kec. Periuk, Kota Tangerang, Banten 15134</t>
+          <t>Jl. Raya Villa Tangerang Indah RT.003/RW.012 Gebang Raya Kec. Periuk Tangerang 15132</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
@@ -4830,17 +4830,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>E684</t>
+          <t>E150</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO SANGIANG TANGERANG</t>
+          <t>ERAFONE CILEGON CENTER MALL</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>CILEGON</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4850,17 +4850,17 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Denny Sanjaya</t>
+          <t>Arif Abdurahman Aziz</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>87880208886</t>
+          <t>81287922331</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Jl. Raya Villa Tangerang Indah RT.003/RW.012 Gebang Raya Kec. Periuk Tangerang 15132</t>
+          <t>Cilegon Center Mall Lt 1 No. 14 , Jl. Ahmad Yani No. 11 Sukmajaya, Kec. Jombang, Kota Cilegon, Banten 42416</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -4875,17 +4875,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>E150</t>
+          <t>E081</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE CILEGON CENTER MALL</t>
+          <t>ERAFONE MALL OF SERANG</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>CILEGON</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -4895,17 +4895,17 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Arif Abdurahman Aziz</t>
+          <t>Andi Saputra</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>81287922331</t>
+          <t>87875027979</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Cilegon Center Mall Lt 1 No. 14 , Jl. Ahmad Yani No. 11 Sukmajaya, Kec. Jombang, Kota Cilegon, Banten 42416</t>
+          <t>Mall of Serang Lantai 1 No. 20, Jl. Akses Tol Serang Tim., Panancangan, Kec. Cipocok Jaya, Kota Serang, Banten 42124</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -4920,12 +4920,12 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>E081</t>
+          <t>E209</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MALL OF SERANG</t>
+          <t>ERAFONE RUKO AHMAD YANI SERANG</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -4940,17 +4940,17 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Andi Saputra</t>
+          <t>Depih Harlan</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>87875027979</t>
+          <t>87701418112</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Mall of Serang Lantai 1 No. 20, Jl. Akses Tol Serang Tim., Panancangan, Kec. Cipocok Jaya, Kota Serang, Banten 42124</t>
+          <t>Jl. Jendral Ahmad Yani No.104 RT RW 001/002 Sumurpecung, Kec. Serang, Kota Serang, Banten 42117</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
@@ -4965,17 +4965,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>E209</t>
+          <t>E194</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO AHMAD YANI SERANG</t>
+          <t>ERAFONE RUKO RANGKASBITUNG</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>RANGKASBITUNG</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -4985,17 +4985,17 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Depih Harlan</t>
+          <t>Fardan Ega Pirmansyah</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>87701418112</t>
+          <t>85694929109</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Jl. Jendral Ahmad Yani No.104 RT RW 001/002 Sumurpecung, Kec. Serang, Kota Serang, Banten 42117</t>
+          <t>Ruko Multatuli Rangkas Bitung, Jl. Multatuli No.95, Muara Ciujung Bar., Kec. Rangkasbitung, Kabupaten Lebak, Banten 42312</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -5010,17 +5010,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>E194</t>
+          <t>E308</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO RANGKASBITUNG</t>
+          <t>ERAFONE RUKO MAYOR SAFEI SERANG</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>RANGKASBITUNG</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -5030,17 +5030,17 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Fardan Ega Pirmansyah</t>
+          <t>Wita Gita Widianti</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>85694929109</t>
+          <t>87786221611</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Ruko Multatuli Rangkas Bitung, Jl. Multatuli No.95, Muara Ciujung Bar., Kec. Rangkasbitung, Kabupaten Lebak, Banten 42312</t>
+          <t>Jalan Mayor Safei Serang , Kel Lontarbaru , Kec Serang , Kota Serang Banten Kode POS 42115</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -5055,17 +5055,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>E308</t>
+          <t>E320</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO MAYOR SAFEI SERANG</t>
+          <t>ERAFONE RUKO PANDEGLANG BANTEN</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>PANDEGLANG</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -5075,17 +5075,17 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Wita Gita Widianti</t>
+          <t>Tubagus Hanifan</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>87786221611</t>
+          <t>85921222664</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Jalan Mayor Safei Serang , Kel Lontarbaru , Kec Serang , Kota Serang Banten Kode POS 42115</t>
+          <t>Jl. Serang Pandeglang, Kel. Pandeglang Kec. Pandeglang, Kab. Pandeglang, Banten kode Pos 42211</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -5100,12 +5100,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>E320</t>
+          <t>E589</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO PANDEGLANG BANTEN</t>
+          <t>ERAFONE RUKO PANIMBANG PANDEGLANG</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -5120,17 +5120,17 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Tubagus Hanifan</t>
+          <t>Ahmad Hidayatulloh</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>85921222664</t>
+          <t>85778211772</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Jl. Serang Pandeglang, Kel. Pandeglang Kec. Pandeglang, Kab. Pandeglang, Banten kode Pos 42211</t>
+          <t>JL. Raya Tanjung - Panimbang, Kp. Padahayu RT 01/04 Ds. Panimbang jaya, Kec. Panimbang Kab. Pandeglang 42281</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -5145,12 +5145,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>E589</t>
+          <t>E499</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO PANIMBANG PANDEGLANG</t>
+          <t>ERAFONE LABUAN PANDEGLANG</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -5165,17 +5165,17 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Ahmad Hidayatulloh</t>
+          <t>Arby Rabiul Tsani</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>85778211772</t>
+          <t>87778810806</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>JL. Raya Tanjung - Panimbang, Kp. Padahayu RT 01/04 Ds. Panimbang jaya, Kec. Panimbang Kab. Pandeglang 42281</t>
+          <t>Jl. Jend. Sudirman No. 99, Muncang Labuan, Kec. Labuang, Pandeglang, Banten 42264</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -5190,17 +5190,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>E499</t>
+          <t>E544</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE LABUAN PANDEGLANG</t>
+          <t>ERAFONE RUKO MULTIBRAND CILEGON</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>PANDEGLANG</t>
+          <t>CILEGON</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -5210,17 +5210,17 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Arby Rabiul Tsani</t>
+          <t>Ahmad Khusnul</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>87778810806</t>
+          <t>895336274142</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Jl. Jend. Sudirman No. 99, Muncang Labuan, Kec. Labuang, Pandeglang, Banten 42264</t>
+          <t>Jl. Simpang Tiga No.13 RT.06 RW.01 Kel. Ramanuju Kec. Purwakarta Cilegon, Banten 42411</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -5235,17 +5235,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>E544</t>
+          <t>E821</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO MULTIBRAND CILEGON</t>
+          <t>ERAFONE MB ANYER</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>CILEGON</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5255,17 +5255,17 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Ahmad Khusnul</t>
+          <t>Ali Rohman</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>895336274142</t>
+          <t>82249001138</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Jl. Simpang Tiga No.13 RT.06 RW.01 Kel. Ramanuju Kec. Purwakarta Cilegon, Banten 42411</t>
+          <t>Jalan Raya Anyer Sirih Kec Anyer Kabupaten Serang Banten 42166</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
@@ -5280,12 +5280,12 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>E821</t>
+          <t>E822</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB ANYER</t>
+          <t>ERAFONE MB KRAGILAN</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -5300,17 +5300,17 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Ali Rohman</t>
+          <t>Marvel Ficky Watuseke</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>82249001138</t>
+          <t>81514421196</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Jalan Raya Anyer Sirih Kec Anyer Kabupaten Serang Banten 42166</t>
+          <t>Jalan raya serang- KM 15, Kragilan, kec Kragilan,Kab Serang BANTEN 42184</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -5325,37 +5325,37 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>E822</t>
+          <t>E833</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB KRAGILAN</t>
+          <t>ERAFONE RANGKASBITUNG 2</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>RANGKASBITUNG</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Marvel Ficky Watuseke</t>
+          <t>M Dede Nurjeli</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>81514421196</t>
+          <t>85894631045</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Jalan raya serang- KM 15, Kragilan, kec Kragilan,Kab Serang BANTEN 42184</t>
+          <t>JL. Sunan kalijaga No.325 Kp. Papanggo RT.01 RW.02 Kel. Cijoro Pasir Rangkasbitung</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
@@ -5370,37 +5370,37 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>E833</t>
+          <t>E879</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RANGKASBITUNG 2</t>
+          <t>ERAFONE MB CIPARE</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>RANGKASBITUNG</t>
+          <t>SERANG</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>M Dede Nurjeli</t>
+          <t>Hendro Wijaya</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>85894631045</t>
+          <t>81906450517</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>JL. Sunan kalijaga No.325 Kp. Papanggo RT.01 RW.02 Kel. Cijoro Pasir Rangkasbitung</t>
+          <t>JL. Raya Pandeglang Sempu, Banten Girang RT.001 RW.017 Kel. Cipare Kec. Serang Kota Serang Banten</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
@@ -5415,37 +5415,37 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>E879</t>
+          <t>M027</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB CIPARE</t>
+          <t>ERAFONE AND MORE CIPUTAT</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>SERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone &amp; More</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>Hendro Wijaya</t>
+          <t>Mochamad Helmi Alatas</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>81906450517</t>
+          <t>85155303034</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>JL. Raya Pandeglang Sempu, Banten Girang RT.001 RW.017 Kel. Cipare Kec. Serang Kota Serang Banten</t>
+          <t>Jl. Dewi Sartika No.12 D, Cipayung, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -5460,12 +5460,12 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>M027</t>
+          <t>E191</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE AND MORE CIPUTAT</t>
+          <t>ERAFONE RUKO SURYA KENCANA PAMULANG</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -5475,22 +5475,22 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Erafone &amp; More</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>Mochamad Helmi Alatas</t>
+          <t>Muhammad Sidik</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>85155303034</t>
+          <t>85770795112</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Jl. Dewi Sartika No.12 D, Cipayung, Kec. Ciputat, Kota Tangerang Selatan, Banten 15411</t>
+          <t>Jl. Surya Kencana No.60, Pamulang Bar., Kec. Pamulang, Kota Tangerang Selatan, Banten 15417</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -5505,12 +5505,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>E191</t>
+          <t>F022</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO SURYA KENCANA PAMULANG</t>
+          <t>ERAFONE 2.5 PAMULANG</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -5525,17 +5525,17 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>Muhammad Sidik</t>
+          <t>Untung</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>85770795112</t>
+          <t>87777192252</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Jl. Surya Kencana No.60, Pamulang Bar., Kec. Pamulang, Kota Tangerang Selatan, Banten 15417</t>
+          <t>Jalan siliwangi no. 2 pondok benda, kec. Pamulang, Banten 15417</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
@@ -5550,12 +5550,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>F022</t>
+          <t>E484</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE 2.5 PAMULANG</t>
+          <t>ERAFONE SERPONG PARADISE WALK</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -5570,17 +5570,17 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Untung</t>
+          <t>Angga Ardian Saputra</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>87777192252</t>
+          <t>89608218065</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Jalan siliwangi no. 2 pondok benda, kec. Pamulang, Banten 15417</t>
+          <t>Jalan Graha Raya Boulevard, Paku Jaya, Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -5595,17 +5595,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>E484</t>
+          <t>E087</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE SERPONG PARADISE WALK</t>
+          <t>ERAFONE ITC BSD</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -5615,17 +5615,17 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Angga Ardian Saputra</t>
+          <t>Aan</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>89608218065</t>
+          <t>81990000098</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Jalan Graha Raya Boulevard, Paku Jaya, Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
+          <t>BSD City, ITC BSD Lantai 3 D3A-6, Jl. Pahlawan Seribu, Lengkong Wetan, Tangerang, Kota Tangerang Selatan, Banten 15321</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -5640,17 +5640,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>E087</t>
+          <t>E941</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE ITC BSD</t>
+          <t>ERAFONE MB RAYA SERPONG</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG</t>
+          <t>TANGERANG SELATAN</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -5660,17 +5660,17 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Aan</t>
+          <t>Ari Firdaus Saputra</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>81990000098</t>
+          <t>85718574849</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>BSD City, ITC BSD Lantai 3 D3A-6, Jl. Pahlawan Seribu, Lengkong Wetan, Tangerang, Kota Tangerang Selatan, Banten 15321</t>
+          <t>Jalan Benda Permai Raya B8/8-B8/9, RT 001, RW 010,Kel/Desa Pondok Benda, Kecamatan Pamulang, Kota Tangerang Selatan, Provinsi Banten</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -5685,12 +5685,12 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>E941</t>
+          <t>E586</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE MB RAYA SERPONG</t>
+          <t>ERAFONE RUKO GRAHA RAYA</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -5705,17 +5705,17 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Ari Firdaus Saputra</t>
+          <t>A Rahman</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>85718574849</t>
+          <t>895326032806</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Jalan Benda Permai Raya B8/8-B8/9, RT 001, RW 010,Kel/Desa Pondok Benda, Kecamatan Pamulang, Kota Tangerang Selatan, Provinsi Banten</t>
+          <t>Jl. Boulevard Graha Raya NO.B15, Paku Jaya, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -5730,12 +5730,12 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>E586</t>
+          <t>E834</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE RUKO GRAHA RAYA</t>
+          <t>ERAFONE KEDAUNG TANGSEL</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -5745,22 +5745,22 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Erafone Multibrand</t>
+          <t>Erafone Franchise</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>A Rahman</t>
+          <t>Samsuri</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>895326032806</t>
+          <t>82213538214</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Jl. Boulevard Graha Raya NO.B15, Paku Jaya, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15220</t>
+          <t>Jl. Pondok Cabe Raya No.9, Kec. Pamulang, Kota Tangerang Selatan, Banten 15418</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -5775,37 +5775,37 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>E834</t>
+          <t>E082</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE KEDAUNG TANGSEL</t>
+          <t>ERAFONE LIVING WORLD ALAM SUTERA</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>TANGERANG SELATAN</t>
+          <t>TANGERANG</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Erafone Franchise</t>
+          <t>Erafone Multibrand</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Samsuri</t>
+          <t>Indra Setiawan</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>82213538214</t>
+          <t>81519578723</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Jl. Pondok Cabe Raya No.9, Kec. Pamulang, Kota Tangerang Selatan, Banten 15418</t>
+          <t>Living World Alam Sutera 1st floor No.30B Jalan Alam Sutera Boulevard Kav. 21, Pakulonan, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15325</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -5820,12 +5820,12 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>E082</t>
+          <t>E088</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>ERAFONE LIVING WORLD ALAM SUTERA</t>
+          <t>ERAFONE AEON MAL BSD CITY</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -5840,65 +5840,20 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Indra Setiawan</t>
+          <t>Gina Tania</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>81519578723</t>
+          <t>85880148262</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Living World Alam Sutera 1st floor No.30B Jalan Alam Sutera Boulevard Kav. 21, Pakulonan, Kec. Serpong Utara, Kota Tangerang Selatan, Banten 15325</t>
+          <t>AEON Mal BSD City Lantai 3 LOT 3-15 Jl. Grand Boulevard BSD City Pagedangan, Kec. Pagedangan, Tangerang, Banten 15345</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
-        <is>
-          <t>Aktif</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>E088</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>ERAFONE AEON MAL BSD CITY</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>TANGERANG</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>Erafone Multibrand</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>Gina Tania</t>
-        </is>
-      </c>
-      <c r="G121" s="2" t="inlineStr">
-        <is>
-          <t>85880148262</t>
-        </is>
-      </c>
-      <c r="H121" s="2" t="inlineStr">
-        <is>
-          <t>AEON Mal BSD City Lantai 3 LOT 3-15 Jl. Grand Boulevard BSD City Pagedangan, Kec. Pagedangan, Tangerang, Banten 15345</t>
-        </is>
-      </c>
-      <c r="I121" s="2" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>

</xml_diff>